<commit_message>
significances graphs with lm models estimates
</commit_message>
<xml_diff>
--- a/results/FD diff x traits.xlsx
+++ b/results/FD diff x traits.xlsx
@@ -12,7 +12,7 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17835"/>
   </bookViews>
   <sheets>
-    <sheet name="FD diff MED" sheetId="2" r:id="rId1"/>
+    <sheet name="FD diff" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -91,7 +91,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -130,8 +130,8 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">

</xml_diff>